<commit_message>
Update .gitignore, enhance chess controller functionality, and remove temporary Excel file
</commit_message>
<xml_diff>
--- a/chess_board.xlsx
+++ b/chess_board.xlsx
@@ -27,18 +27,54 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
-  <si>
-    <t>Nước đi của bạn</t>
-  </si>
-  <si>
-    <t>Nút/Ô trạng thái gửi nước đi.</t>
-  </si>
-  <si>
-    <t>Trạng thái bàn cờ</t>
-  </si>
-  <si>
-    <t>Nước đi vừa qua của Stockfish.</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="24">
+  <si>
+    <t>♜</t>
+  </si>
+  <si>
+    <t>♞</t>
+  </si>
+  <si>
+    <t>♝</t>
+  </si>
+  <si>
+    <t>♛</t>
+  </si>
+  <si>
+    <t>♚</t>
+  </si>
+  <si>
+    <t>Nhập nước đi của bạn và nhấn Enter</t>
+  </si>
+  <si>
+    <t>&lt;-- Nhập "reset"</t>
+  </si>
+  <si>
+    <t>♟</t>
+  </si>
+  <si>
+    <t>Đến lượt bạn (Trắng).</t>
+  </si>
+  <si>
+    <t>♙</t>
+  </si>
+  <si>
+    <t>Nước đi của Stockfish</t>
+  </si>
+  <si>
+    <t>♖</t>
+  </si>
+  <si>
+    <t>♘</t>
+  </si>
+  <si>
+    <t>♗</t>
+  </si>
+  <si>
+    <t>♕</t>
+  </si>
+  <si>
+    <t>♔</t>
   </si>
   <si>
     <t>a</t>
@@ -75,7 +111,7 @@
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="22">
+  <fonts count="23">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -85,7 +121,7 @@
     </font>
     <font>
       <b/>
-      <sz val="11"/>
+      <sz val="22"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
@@ -93,7 +129,15 @@
     </font>
     <font>
       <b/>
-      <sz val="11"/>
+      <sz val="22"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="22"/>
       <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <charset val="134"/>
@@ -244,7 +288,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="35">
+  <fills count="34">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -374,12 +418,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -591,154 +629,166 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -1271,46 +1321,81 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="B3:L11"/>
+  <dimension ref="B3:O11"/>
   <sheetFormatPr defaultColWidth="8.72727272727273" defaultRowHeight="14.5"/>
   <cols>
     <col min="2" max="10" width="6.63636363636364" customWidth="1"/>
-    <col min="12" max="12" width="17.5454545454545" customWidth="1"/>
+    <col min="12" max="12" width="35.0727272727273" customWidth="1"/>
+    <col min="15" max="15" width="17.6454545454545" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" ht="36" customHeight="1" spans="2:12">
+    <row r="3" ht="36" customHeight="1" spans="2:15">
       <c r="B3" s="1">
         <v>8</v>
       </c>
-      <c r="C3" s="2"/>
-      <c r="D3" s="3"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="3"/>
-      <c r="G3" s="2"/>
-      <c r="H3" s="3"/>
-      <c r="I3" s="2"/>
-      <c r="J3" s="3"/>
+      <c r="C3" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>0</v>
+      </c>
       <c r="L3" s="4" t="s">
-        <v>0</v>
+        <v>5</v>
+      </c>
+      <c r="N3" s="5"/>
+      <c r="O3" s="4" t="s">
+        <v>6</v>
       </c>
     </row>
-    <row r="4" ht="36" customHeight="1" spans="2:12">
+    <row r="4" ht="36" customHeight="1" spans="2:15">
       <c r="B4" s="1">
         <v>7</v>
       </c>
-      <c r="C4" s="3"/>
-      <c r="D4" s="2"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="2"/>
-      <c r="G4" s="3"/>
-      <c r="H4" s="2"/>
-      <c r="I4" s="3"/>
-      <c r="J4" s="2"/>
-      <c r="L4" t="s">
-        <v>1</v>
-      </c>
+      <c r="C4" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="L4" s="5"/>
     </row>
-    <row r="5" ht="36" customHeight="1" spans="2:12">
+    <row r="5" ht="36" customHeight="1" spans="2:15">
       <c r="B5" s="1">
         <v>6</v>
       </c>
@@ -1323,7 +1408,7 @@
       <c r="I5" s="2"/>
       <c r="J5" s="3"/>
     </row>
-    <row r="6" ht="36" customHeight="1" spans="2:12">
+    <row r="6" ht="36" customHeight="1" spans="2:15">
       <c r="B6" s="1">
         <v>5</v>
       </c>
@@ -1335,11 +1420,11 @@
       <c r="H6" s="2"/>
       <c r="I6" s="3"/>
       <c r="J6" s="2"/>
-      <c r="L6" t="s">
-        <v>2</v>
+      <c r="L6" s="6" t="s">
+        <v>8</v>
       </c>
     </row>
-    <row r="7" ht="36" customHeight="1" spans="2:12">
+    <row r="7" ht="36" customHeight="1" spans="2:15">
       <c r="B7" s="1">
         <v>4</v>
       </c>
@@ -1352,7 +1437,7 @@
       <c r="I7" s="2"/>
       <c r="J7" s="3"/>
     </row>
-    <row r="8" ht="36" customHeight="1" spans="2:12">
+    <row r="8" ht="36" customHeight="1" spans="2:15">
       <c r="B8" s="1">
         <v>3</v>
       </c>
@@ -1364,60 +1449,94 @@
       <c r="H8" s="2"/>
       <c r="I8" s="3"/>
       <c r="J8" s="2"/>
-      <c r="L8" t="s">
-        <v>3</v>
-      </c>
+      <c r="L8" s="5"/>
     </row>
-    <row r="9" ht="36" customHeight="1" spans="2:12">
+    <row r="9" ht="36" customHeight="1" spans="2:15">
       <c r="B9" s="1">
         <v>2</v>
       </c>
-      <c r="C9" s="2"/>
-      <c r="D9" s="3"/>
-      <c r="E9" s="2"/>
-      <c r="F9" s="3"/>
-      <c r="G9" s="2"/>
-      <c r="H9" s="3"/>
-      <c r="I9" s="2"/>
-      <c r="J9" s="3"/>
+      <c r="C9" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="D9" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="F9" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="G9" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="H9" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="I9" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="J9" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="L9" s="4" t="s">
+        <v>10</v>
+      </c>
     </row>
-    <row r="10" ht="36" customHeight="1" spans="2:12">
+    <row r="10" ht="36" customHeight="1" spans="2:15">
       <c r="B10" s="1">
         <v>1</v>
       </c>
-      <c r="C10" s="3"/>
-      <c r="D10" s="2"/>
-      <c r="E10" s="3"/>
-      <c r="F10" s="2"/>
-      <c r="G10" s="3"/>
-      <c r="H10" s="2"/>
-      <c r="I10" s="3"/>
-      <c r="J10" s="2"/>
+      <c r="C10" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="E10" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="F10" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="G10" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="H10" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="I10" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="J10" s="7" t="s">
+        <v>11</v>
+      </c>
     </row>
-    <row r="11" ht="40" customHeight="1" spans="2:12">
-      <c r="C11" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="D11" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="E11" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="F11" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="G11" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="H11" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="I11" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="J11" s="5" t="s">
-        <v>11</v>
+    <row r="11" ht="40" customHeight="1" spans="2:15">
+      <c r="B11" s="9"/>
+      <c r="C11" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="I11" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="J11" s="1" t="s">
+        <v>23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>